<commit_message>
Final Changes for Now
</commit_message>
<xml_diff>
--- a/Sprint Requirement Plan.xlsx
+++ b/Sprint Requirement Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\LudusRecommender\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7779BC30-AECC-4FDA-B7A4-CD23D7CD278E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A12B35-D18C-4F93-8D78-5B8B04A2380A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="3165" windowWidth="26940" windowHeight="11295" xr2:uid="{B75432DC-D21B-4DDC-BFE0-85395F7A9756}"/>
+    <workbookView xWindow="255" yWindow="3615" windowWidth="26940" windowHeight="11295" xr2:uid="{B75432DC-D21B-4DDC-BFE0-85395F7A9756}"/>
   </bookViews>
   <sheets>
     <sheet name="FR" sheetId="1" r:id="rId1"/>
@@ -768,16 +768,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1102,10 +1102,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="4" t="s">
@@ -1164,10 +1164,10 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="26.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="7"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="4" t="s">
@@ -1226,13 +1226,13 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="26.25">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="9"/>
+      <c r="B17" s="8"/>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1240,7 +1240,7 @@
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1248,7 +1248,7 @@
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1316,10 +1316,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="7"/>
+      <c r="B1" s="9"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="4" t="s">
@@ -1346,10 +1346,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="26.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="7"/>
+      <c r="B5" s="9"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
@@ -1384,10 +1384,10 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="26.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="10"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="3" t="s">

</xml_diff>

<commit_message>
Updated Sprint Requirement Plan
</commit_message>
<xml_diff>
--- a/Sprint Requirement Plan.xlsx
+++ b/Sprint Requirement Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\LudusRecommender\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A12B35-D18C-4F93-8D78-5B8B04A2380A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FF6144-E06F-4651-A4B2-8750D9EE71D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="255" yWindow="3615" windowWidth="26940" windowHeight="11295" xr2:uid="{B75432DC-D21B-4DDC-BFE0-85395F7A9756}"/>
   </bookViews>
@@ -1256,7 +1256,7 @@
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1264,7 +1264,7 @@
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1272,7 +1272,7 @@
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>50</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1280,7 +1280,7 @@
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B24" s="1" t="s">

</xml_diff>